<commit_message>
Update ArduinoUnoQ BOM and schematic
</commit_message>
<xml_diff>
--- a/PCBA/BOM.xlsx
+++ b/PCBA/BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LuwuProject\ArduinoUnoQ\ArduinoUnoQV1\Arduino载板开源文件\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC53DB41-C1E1-4968-84D8-22EC13D0CEFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A1F1E57-9561-45EC-9565-061205813242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="3945" windowWidth="38640" windowHeight="21120" xr2:uid="{826F304B-56DA-4286-AE05-E386D77AFD3B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="85">
   <si>
     <t>Comment</t>
   </si>
@@ -101,24 +101,12 @@
     <t>CONN-TH_2P-P2.50_ZX-XH2.54-2PWZ</t>
   </si>
   <si>
-    <t>LED/G</t>
-  </si>
-  <si>
     <t>Typical INFRARED GaAs LED</t>
   </si>
   <si>
-    <t>D1</t>
-  </si>
-  <si>
     <t>D_SOD_523</t>
   </si>
   <si>
-    <t>LED/Y</t>
-  </si>
-  <si>
-    <t>D2</t>
-  </si>
-  <si>
     <t>LED/R</t>
   </si>
   <si>
@@ -215,97 +203,100 @@
     <t>Resistor</t>
   </si>
   <si>
+    <t>R0603</t>
+  </si>
+  <si>
+    <t>4.7K/±1%</t>
+  </si>
+  <si>
+    <t>1k/±1%</t>
+  </si>
+  <si>
+    <t>3.3K/±1%</t>
+  </si>
+  <si>
+    <t>R10</t>
+  </si>
+  <si>
+    <t>20K/±1%</t>
+  </si>
+  <si>
+    <t>R11</t>
+  </si>
+  <si>
+    <t>SN74LVC1G126</t>
+  </si>
+  <si>
+    <t>输出缓冲器</t>
+  </si>
+  <si>
+    <t>SN1</t>
+  </si>
+  <si>
+    <t>SOT_23_5</t>
+  </si>
+  <si>
+    <t>SN74LVC1G125</t>
+  </si>
+  <si>
+    <t>SN2</t>
+  </si>
+  <si>
+    <t>SS-12D06L5</t>
+  </si>
+  <si>
+    <t>电路结构:单刀双掷;安装方式:-;开关颜色:黑色;额定电流:3A;额定电压:125V;工作寿命:1万次;</t>
+  </si>
+  <si>
+    <t>SW1</t>
+  </si>
+  <si>
+    <t>SW-TH_3P-P4.70_L11.1-W12.7</t>
+  </si>
+  <si>
+    <t>QMI8658A</t>
+  </si>
+  <si>
+    <t>六轴陀螺仪  陀螺仪量程(MAX) ±2048dps  加速度计量程(MAX) ±16g</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>LGA-14_L3.0-W2.5-P0.50-TL</t>
+  </si>
+  <si>
+    <t>h7651-50pr</t>
+  </si>
+  <si>
+    <t>输出极性:正极;工作电压:8.5V;输出电压:5V;输出电流:1A;电源纹波抑制比(PSRR):-;输出类型:固定;</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>292253-3</t>
+  </si>
+  <si>
+    <t>插针结构:1x3P;间距:2mm;安装方式:弯插;总PIN数:3P;排数:1;每排PIN数:3;额定电流:4A;触头材质:黄铜;触头镀层:锡;工作温度:-40℃~+105℃;</t>
+  </si>
+  <si>
+    <t>U3, U4, U5</t>
+  </si>
+  <si>
+    <t>CONN-TH_3P-P2.00_TE_292253-3</t>
+  </si>
+  <si>
+    <t>R2, R3, R4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>R1, R5, R8</t>
-  </si>
-  <si>
-    <t>R0603</t>
-  </si>
-  <si>
-    <t>4.7K/±1%</t>
-  </si>
-  <si>
-    <t>R2, R3, R4</t>
-  </si>
-  <si>
-    <t>1k/±1%</t>
-  </si>
-  <si>
-    <t>R6, R7, R9</t>
-  </si>
-  <si>
-    <t>3.3K/±1%</t>
-  </si>
-  <si>
-    <t>R10</t>
-  </si>
-  <si>
-    <t>20K/±1%</t>
-  </si>
-  <si>
-    <t>R11</t>
-  </si>
-  <si>
-    <t>SN74LVC1G126</t>
-  </si>
-  <si>
-    <t>输出缓冲器</t>
-  </si>
-  <si>
-    <t>SN1</t>
-  </si>
-  <si>
-    <t>SOT_23_5</t>
-  </si>
-  <si>
-    <t>SN74LVC1G125</t>
-  </si>
-  <si>
-    <t>SN2</t>
-  </si>
-  <si>
-    <t>SS-12D06L5</t>
-  </si>
-  <si>
-    <t>电路结构:单刀双掷;安装方式:-;开关颜色:黑色;额定电流:3A;额定电压:125V;工作寿命:1万次;</t>
-  </si>
-  <si>
-    <t>SW1</t>
-  </si>
-  <si>
-    <t>SW-TH_3P-P4.70_L11.1-W12.7</t>
-  </si>
-  <si>
-    <t>QMI8658A</t>
-  </si>
-  <si>
-    <t>六轴陀螺仪  陀螺仪量程(MAX) ±2048dps  加速度计量程(MAX) ±16g</t>
-  </si>
-  <si>
-    <t>U1</t>
-  </si>
-  <si>
-    <t>LGA-14_L3.0-W2.5-P0.50-TL</t>
-  </si>
-  <si>
-    <t>h7651-50pr</t>
-  </si>
-  <si>
-    <t>输出极性:正极;工作电压:8.5V;输出电压:5V;输出电流:1A;电源纹波抑制比(PSRR):-;输出类型:固定;</t>
-  </si>
-  <si>
-    <t>U2</t>
-  </si>
-  <si>
-    <t>292253-3</t>
-  </si>
-  <si>
-    <t>插针结构:1x3P;间距:2mm;安装方式:弯插;总PIN数:3P;排数:1;每排PIN数:3;额定电流:4A;触头材质:黄铜;触头镀层:锡;工作温度:-40℃~+105℃;</t>
-  </si>
-  <si>
-    <t>U3, U4, U5</t>
-  </si>
-  <si>
-    <t>CONN-TH_3P-P2.00_TE_292253-3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>R9</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -722,12 +713,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B08E26E6-B0E0-43B2-A9DD-9C051998C4C9}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
-    <col min="2" max="2" width="56.58203125" customWidth="1"/>
-    <col min="3" max="5" width="17.33203125" customWidth="1"/>
+    <col min="2" max="2" width="92.08203125" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" customWidth="1"/>
+    <col min="4" max="4" width="42.6640625" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -834,19 +827,19 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="E7" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -854,13 +847,13 @@
         <v>24</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E8" s="1">
         <v>1</v>
@@ -868,33 +861,33 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="E9" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E10" s="1">
         <v>1</v>
@@ -902,104 +895,104 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E11" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E12" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E13" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E14" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E15" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>53</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>55</v>
-      </c>
       <c r="E16" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -1007,13 +1000,13 @@
         <v>56</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>58</v>
+        <v>84</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="E17" s="1">
         <v>3</v>
@@ -1021,50 +1014,50 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="E18" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="E19" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>59</v>
       </c>
       <c r="E20" s="1">
         <v>1</v>
@@ -1072,16 +1065,16 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="D21" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="E21" s="1">
         <v>1</v>
@@ -1089,16 +1082,16 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="E22" s="1">
         <v>1</v>
@@ -1106,16 +1099,16 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E23" s="1">
         <v>1</v>
@@ -1123,16 +1116,16 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="E24" s="1">
         <v>1</v>
@@ -1152,40 +1145,6 @@
         <v>81</v>
       </c>
       <c r="E25" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E26" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E27" s="1">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ArduinoUnoQ hardware design files
</commit_message>
<xml_diff>
--- a/PCBA/BOM.xlsx
+++ b/PCBA/BOM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LuwuProject\ArduinoUnoQ\ArduinoUnoQV1\Arduino载板开源文件\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LuwuProject\ArduinoUnoQ\ArduinoUnoQV1\Project Outputs for ArduinoUnoQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A1F1E57-9561-45EC-9565-061205813242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B886406D-7AEE-4E6F-B309-027670E25964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="3945" windowWidth="38640" windowHeight="21120" xr2:uid="{826F304B-56DA-4286-AE05-E386D77AFD3B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{60F18D17-E70B-4507-8B15-82C9613171DE}"/>
   </bookViews>
   <sheets>
     <sheet name="ArduinoUnoQ" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="86">
   <si>
     <t>Comment</t>
   </si>
@@ -71,9 +71,6 @@
     <t>100nF/25V</t>
   </si>
   <si>
-    <t>0603贴片电容，±10%，50V, 贴片电容</t>
-  </si>
-  <si>
     <t>C2, C4, C5, C9, C11</t>
   </si>
   <si>
@@ -101,18 +98,18 @@
     <t>CONN-TH_2P-P2.50_ZX-XH2.54-2PWZ</t>
   </si>
   <si>
+    <t>LED/R</t>
+  </si>
+  <si>
     <t>Typical INFRARED GaAs LED</t>
   </si>
   <si>
+    <t>D3, D4</t>
+  </si>
+  <si>
     <t>D_SOD_523</t>
   </si>
   <si>
-    <t>LED/R</t>
-  </si>
-  <si>
-    <t>D3, D4</t>
-  </si>
-  <si>
     <t>kh-dc-007b-2.1g</t>
   </si>
   <si>
@@ -161,10 +158,10 @@
     <t>HDR-TH_8P-P2.54-V-M</t>
   </si>
   <si>
-    <t>Header 3</t>
-  </si>
-  <si>
-    <t>Header, 3-Pin</t>
+    <t>mx1.25 1*3P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1x3P 间距:1.25mm 直插 </t>
   </si>
   <si>
     <t>P1, P2, P3</t>
@@ -176,7 +173,7 @@
     <t>BC807</t>
   </si>
   <si>
-    <t>三极管BJT</t>
+    <t>hfe=250~600 PNP 电流:500mA 电压:45V</t>
   </si>
   <si>
     <t>Q1</t>
@@ -200,7 +197,10 @@
     <t>10K/±1%</t>
   </si>
   <si>
-    <t>Resistor</t>
+    <t>厚膜电阻  ±1% 100mW</t>
+  </si>
+  <si>
+    <t>R1, R5, R8</t>
   </si>
   <si>
     <t>R0603</t>
@@ -209,7 +209,16 @@
     <t>4.7K/±1%</t>
   </si>
   <si>
-    <t>1k/±1%</t>
+    <t>R2, R3, R4</t>
+  </si>
+  <si>
+    <t>1K/±1%</t>
+  </si>
+  <si>
+    <t>厚膜电阻 ±1% 100mW</t>
+  </si>
+  <si>
+    <t>R9</t>
   </si>
   <si>
     <t>3.3K/±1%</t>
@@ -227,7 +236,7 @@
     <t>SN74LVC1G126</t>
   </si>
   <si>
-    <t>输出缓冲器</t>
+    <t>三态输出，单路总线缓冲门</t>
   </si>
   <si>
     <t>SN1</t>
@@ -239,6 +248,9 @@
     <t>SN74LVC1G125</t>
   </si>
   <si>
+    <t>单总线缓冲门，带三态输出</t>
+  </si>
+  <si>
     <t>SN2</t>
   </si>
   <si>
@@ -285,18 +297,6 @@
   </si>
   <si>
     <t>CONN-TH_3P-P2.00_TE_292253-3</t>
-  </si>
-  <si>
-    <t>R2, R3, R4</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>R1, R5, R8</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>R9</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -367,17 +367,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -712,439 +712,438 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B08E26E6-B0E0-43B2-A9DD-9C051998C4C9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B937F53F-E96F-415C-B681-EF2E71E4CE2B}">
   <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
-    <col min="2" max="2" width="92.08203125" customWidth="1"/>
-    <col min="3" max="3" width="17.33203125" customWidth="1"/>
-    <col min="4" max="4" width="42.6640625" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="30.5" customWidth="1"/>
+    <col min="2" max="2" width="70.75" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="4" max="5" width="17.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="4">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="B4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="E4" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="C5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="E5" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="42" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="E7" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="28" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="1">
+      <c r="B8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="42" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="42" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="42" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E10" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" s="2" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="1">
+      <c r="B13" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="42" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E15" s="4">
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E13" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" s="2" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E16" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E17" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E18" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E20" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="28" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E22" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="28" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E23" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="42" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E14" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="E24" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="28" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E15" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E16" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C17" s="2" t="s">
+      <c r="C25" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E17" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E18" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E19" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E20" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E21" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E22" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E23" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E24" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="E25" s="1">
+      <c r="D25" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E25" s="4">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ArduinoUnoQ schematic and BOM and simplify servo notice
</commit_message>
<xml_diff>
--- a/PCBA/BOM.xlsx
+++ b/PCBA/BOM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LuwuProject\ArduinoUnoQ\ArduinoUnoQV1\Arduino载板开源文件\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LuwuProject\ArduinoUnoQ\ArduinoUnoQV1\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A1F1E57-9561-45EC-9565-061205813242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10043800-024F-49F6-9ACB-8F53AA09AEBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="3945" windowWidth="38640" windowHeight="21120" xr2:uid="{826F304B-56DA-4286-AE05-E386D77AFD3B}"/>
+    <workbookView xWindow="-38520" yWindow="3945" windowWidth="38640" windowHeight="21120" xr2:uid="{60F18D17-E70B-4507-8B15-82C9613171DE}"/>
   </bookViews>
   <sheets>
     <sheet name="ArduinoUnoQ" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="86">
   <si>
     <t>Comment</t>
   </si>
@@ -71,9 +71,6 @@
     <t>100nF/25V</t>
   </si>
   <si>
-    <t>0603贴片电容，±10%，50V, 贴片电容</t>
-  </si>
-  <si>
     <t>C2, C4, C5, C9, C11</t>
   </si>
   <si>
@@ -101,18 +98,18 @@
     <t>CONN-TH_2P-P2.50_ZX-XH2.54-2PWZ</t>
   </si>
   <si>
+    <t>LED/R</t>
+  </si>
+  <si>
     <t>Typical INFRARED GaAs LED</t>
   </si>
   <si>
+    <t>D3, D4</t>
+  </si>
+  <si>
     <t>D_SOD_523</t>
   </si>
   <si>
-    <t>LED/R</t>
-  </si>
-  <si>
-    <t>D3, D4</t>
-  </si>
-  <si>
     <t>kh-dc-007b-2.1g</t>
   </si>
   <si>
@@ -161,10 +158,10 @@
     <t>HDR-TH_8P-P2.54-V-M</t>
   </si>
   <si>
-    <t>Header 3</t>
-  </si>
-  <si>
-    <t>Header, 3-Pin</t>
+    <t>mx1.25 1*3P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1x3P 间距:1.25mm 直插 </t>
   </si>
   <si>
     <t>P1, P2, P3</t>
@@ -176,7 +173,7 @@
     <t>BC807</t>
   </si>
   <si>
-    <t>三极管BJT</t>
+    <t>hfe=250~600 PNP 电流:500mA 电压:45V</t>
   </si>
   <si>
     <t>Q1</t>
@@ -200,7 +197,10 @@
     <t>10K/±1%</t>
   </si>
   <si>
-    <t>Resistor</t>
+    <t>厚膜电阻  ±1% 100mW</t>
+  </si>
+  <si>
+    <t>R1, R5, R8</t>
   </si>
   <si>
     <t>R0603</t>
@@ -209,7 +209,16 @@
     <t>4.7K/±1%</t>
   </si>
   <si>
-    <t>1k/±1%</t>
+    <t>R2, R3, R4</t>
+  </si>
+  <si>
+    <t>1K/±1%</t>
+  </si>
+  <si>
+    <t>厚膜电阻 ±1% 100mW</t>
+  </si>
+  <si>
+    <t>R9</t>
   </si>
   <si>
     <t>3.3K/±1%</t>
@@ -227,7 +236,7 @@
     <t>SN74LVC1G126</t>
   </si>
   <si>
-    <t>输出缓冲器</t>
+    <t>三态输出，单路总线缓冲门</t>
   </si>
   <si>
     <t>SN1</t>
@@ -239,6 +248,9 @@
     <t>SN74LVC1G125</t>
   </si>
   <si>
+    <t>单总线缓冲门，带三态输出</t>
+  </si>
+  <si>
     <t>SN2</t>
   </si>
   <si>
@@ -266,12 +278,6 @@
     <t>LGA-14_L3.0-W2.5-P0.50-TL</t>
   </si>
   <si>
-    <t>h7651-50pr</t>
-  </si>
-  <si>
-    <t>输出极性:正极;工作电压:8.5V;输出电压:5V;输出电流:1A;电源纹波抑制比(PSRR):-;输出类型:固定;</t>
-  </si>
-  <si>
     <t>U2</t>
   </si>
   <si>
@@ -287,15 +293,11 @@
     <t>CONN-TH_3P-P2.00_TE_292253-3</t>
   </si>
   <si>
-    <t>R2, R3, R4</t>
+    <t>HT7550-1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>R1, R5, R8</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>R9</t>
+    <t>线性稳压器(LDO),5V 150mA 30V</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -367,17 +369,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -712,439 +714,438 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B08E26E6-B0E0-43B2-A9DD-9C051998C4C9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B937F53F-E96F-415C-B681-EF2E71E4CE2B}">
   <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
-    <col min="2" max="2" width="92.08203125" customWidth="1"/>
-    <col min="3" max="3" width="17.33203125" customWidth="1"/>
-    <col min="4" max="4" width="42.6640625" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="30.5" customWidth="1"/>
+    <col min="2" max="2" width="70.75" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="4" max="5" width="17.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="4">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="B4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="E4" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="C5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="E5" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="42" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="E7" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="28" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="1">
+      <c r="B8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="42" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="42" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="42" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E10" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" s="2" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="1">
+      <c r="B13" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="42" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E15" s="4">
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E13" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" s="2" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E16" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E17" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E18" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E20" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="28" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E22" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="28" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E23" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="42" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E14" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="E24" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="28" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E15" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E16" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E17" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E18" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E19" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E20" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E21" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E22" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E23" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E24" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="E25" s="1">
+      <c r="E25" s="4">
         <v>3</v>
       </c>
     </row>

</xml_diff>